<commit_message>
Migrating to Laptop post theft
</commit_message>
<xml_diff>
--- a/BOM/Parts List and Cost Analysis.xlsx
+++ b/BOM/Parts List and Cost Analysis.xlsx
@@ -1,28 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dcdf7eb514dfaeec/Projects/Microgravity-Press-Washing-Machine/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BDCCF2F-CD62-4976-945E-343FBA828B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{1BDCCF2F-CD62-4976-945E-343FBA828B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75C551CA-006B-4DDF-8BB2-E2DC225DC745}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts &amp; Assembly List" sheetId="1" r:id="rId1"/>
     <sheet name="Part Count and Cost Estimate" sheetId="5" r:id="rId2"/>
     <sheet name="Tools Needed" sheetId="2" r:id="rId3"/>
     <sheet name="Part Catagory Key" sheetId="3" r:id="rId4"/>
-    <sheet name="Operational Consumables" sheetId="4" r:id="rId5"/>
+    <sheet name="Temp" sheetId="6" r:id="rId5"/>
+    <sheet name="Operational Consumables" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parts &amp; Assembly List'!$A$2:$M$463</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="322">
   <si>
     <t>$/kg</t>
   </si>
@@ -1010,6 +1011,24 @@
   </si>
   <si>
     <t>Smallest off the shelf latch I could find. I feel like a more purpose built construction could be found, but I haven't been able to find anything</t>
+  </si>
+  <si>
+    <t>https://www.mcmaster.com/9573K16/</t>
+  </si>
+  <si>
+    <t>New Springs for Reservoir Piston</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/gp/product/B0B6SF3PHK?smid=A3E0SBPIY1LXW8&amp;th=1</t>
+  </si>
+  <si>
+    <t>Pressure Regulator Valve</t>
+  </si>
+  <si>
+    <t>https://www.mcmaster.com/91257A553/</t>
+  </si>
+  <si>
+    <t>Bolt</t>
   </si>
 </sst>
 </file>
@@ -1445,16 +1464,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O446"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="50.3984375" customWidth="1"/>
-    <col min="12" max="12" width="20.59765625" customWidth="1"/>
-    <col min="13" max="13" width="10.86328125" style="3" customWidth="1"/>
-    <col min="15" max="15" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.44140625" customWidth="1"/>
+    <col min="12" max="12" width="20.5546875" customWidth="1"/>
+    <col min="13" max="13" width="10.88671875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="F1" t="s">
         <v>79</v>
       </c>
@@ -1462,7 +1481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1503,7 +1522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>49</v>
       </c>
@@ -1548,7 +1567,7 @@
       </c>
       <c r="O3" s="8"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>49</v>
       </c>
@@ -1586,7 +1605,7 @@
         <v>45632.707033796294</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>49</v>
       </c>
@@ -1624,7 +1643,7 @@
         <v>45642.655523842594</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>49</v>
       </c>
@@ -1662,7 +1681,7 @@
         <v>45642.655523842594</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>49</v>
       </c>
@@ -1703,7 +1722,7 @@
         <v>45632.714402083337</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>63</v>
       </c>
@@ -1744,7 +1763,7 @@
         <v>45632.711294791668</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>49</v>
       </c>
@@ -1785,7 +1804,7 @@
         <v>45632.720302083333</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>49</v>
       </c>
@@ -1826,7 +1845,7 @@
         <v>45794.977847569447</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>49</v>
       </c>
@@ -1865,7 +1884,7 @@
         <v>45794.977792361111</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>49</v>
       </c>
@@ -1903,7 +1922,7 @@
         <v>45643.561000578702</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>49</v>
       </c>
@@ -1941,7 +1960,7 @@
         <v>45694.801739120368</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>49</v>
       </c>
@@ -1979,7 +1998,7 @@
         <v>45632.721292361108</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>49</v>
       </c>
@@ -2017,7 +2036,7 @@
         <v>45794.570570717595</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>49</v>
       </c>
@@ -2055,7 +2074,7 @@
         <v>45794.571933912041</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>49</v>
       </c>
@@ -2093,7 +2112,7 @@
         <v>45794.746052199072</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>49</v>
       </c>
@@ -2131,7 +2150,7 @@
         <v>45643.711436689817</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>49</v>
       </c>
@@ -2172,7 +2191,7 @@
         <v>45642.687478356478</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>49</v>
       </c>
@@ -2210,7 +2229,7 @@
         <v>45642.535365509262</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>49</v>
       </c>
@@ -2251,7 +2270,7 @@
         <v>45643.562765972223</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>49</v>
       </c>
@@ -2289,7 +2308,7 @@
         <v>45643.711616666667</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>49</v>
       </c>
@@ -2327,7 +2346,7 @@
         <v>45642.648433912036</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>49</v>
       </c>
@@ -2368,7 +2387,7 @@
         <v>45642.647163541667</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>49</v>
       </c>
@@ -2406,7 +2425,7 @@
         <v>45643.882129398145</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>49</v>
       </c>
@@ -2444,7 +2463,7 @@
         <v>45684.7621349537</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>49</v>
       </c>
@@ -2485,7 +2504,7 @@
         <v>45646.886742939816</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>49</v>
       </c>
@@ -2523,7 +2542,7 @@
         <v>45746.871895486111</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>49</v>
       </c>
@@ -2561,7 +2580,7 @@
         <v>45646.890947222222</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>49</v>
       </c>
@@ -2600,7 +2619,7 @@
         <v>45794.746517013889</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>49</v>
       </c>
@@ -2639,7 +2658,7 @@
         <v>45696.724602314818</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>49</v>
       </c>
@@ -2680,7 +2699,7 @@
         <v>45809.893460300926</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>49</v>
       </c>
@@ -2721,7 +2740,7 @@
         <v>45794.948679976849</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>49</v>
       </c>
@@ -2759,7 +2778,7 @@
         <v>45794.94740902778</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>49</v>
       </c>
@@ -2800,7 +2819,7 @@
         <v>45794.991633564816</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>49</v>
       </c>
@@ -2841,7 +2860,7 @@
         <v>45699.639482407409</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>49</v>
       </c>
@@ -2882,7 +2901,7 @@
         <v>45794.992589236113</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>49</v>
       </c>
@@ -2920,7 +2939,7 @@
         <v>45699.639453356482</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>49</v>
       </c>
@@ -2961,7 +2980,7 @@
         <v>45759.449647222224</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>49</v>
       </c>
@@ -2999,7 +3018,7 @@
         <v>45794.930470833337</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>49</v>
       </c>
@@ -3036,7 +3055,7 @@
         <v>45795.009833217591</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>49</v>
       </c>
@@ -3074,7 +3093,7 @@
         <v>45759.449647222224</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>49</v>
       </c>
@@ -3115,7 +3134,7 @@
         <v>45794.917324652779</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>49</v>
       </c>
@@ -3153,7 +3172,7 @@
         <v>45794.914960069444</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>49</v>
       </c>
@@ -3191,7 +3210,7 @@
         <v>45794.89084699074</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>49</v>
       </c>
@@ -3232,7 +3251,7 @@
         <v>45794.918360300922</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>49</v>
       </c>
@@ -3273,7 +3292,7 @@
         <v>45794.918360300922</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>49</v>
       </c>
@@ -3311,7 +3330,7 @@
         <v>45794.573409143515</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>49</v>
       </c>
@@ -3346,10 +3365,10 @@
       </c>
       <c r="M49" s="3" cm="1">
         <f t="array" aca="1" ref="M49" ca="1">IF(OR(CELL("address")=CELL("address",A49),CELL("address")=CELL("address",B49),CELL("address")=CELL("address",C49),CELL("address")=CELL("address",D49),CELL("address")=CELL("address",E49),CELL("address")=CELL("address",F49),CELL("address")=CELL("address",G49),CELL("address")=CELL("address",H49),CELL("address")=CELL("address",I49)),NOW(),M49)</f>
-        <v>46026.352704398145</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.45">
+        <v>46051.8697994213</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>49</v>
       </c>
@@ -3387,7 +3406,7 @@
         <v>45661.896769675928</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>49</v>
       </c>
@@ -3425,7 +3444,7 @@
         <v>45646.883798726849</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>49</v>
       </c>
@@ -3463,7 +3482,7 @@
         <v>45646.883798726849</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>49</v>
       </c>
@@ -3501,7 +3520,7 @@
         <v>45646.883798726849</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>49</v>
       </c>
@@ -3542,7 +3561,7 @@
         <v>45795.01019872685</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
         <v>49</v>
       </c>
@@ -3583,7 +3602,7 @@
         <v>45661.891742361113</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>63</v>
       </c>
@@ -3621,7 +3640,7 @@
         <v>45661.895691898149</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>49</v>
       </c>
@@ -3659,7 +3678,7 @@
         <v>45646.883798726849</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>49</v>
       </c>
@@ -3697,7 +3716,7 @@
         <v>45646.883798726849</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>49</v>
       </c>
@@ -3735,7 +3754,7 @@
         <v>45795.010351851852</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>178</v>
       </c>
@@ -3773,7 +3792,7 @@
         <v>45795.010864004631</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>63</v>
       </c>
@@ -3811,7 +3830,7 @@
         <v>45646.897749305557</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>49</v>
       </c>
@@ -3849,7 +3868,7 @@
         <v>45661.896488078703</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>49</v>
       </c>
@@ -3890,7 +3909,7 @@
         <v>45646.883798726849</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>49</v>
       </c>
@@ -3931,7 +3950,7 @@
         <v>45646.883798726849</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
         <v>49</v>
       </c>
@@ -3970,7 +3989,7 @@
         <v>45794.749220138889</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
         <v>49</v>
       </c>
@@ -4008,7 +4027,7 @@
         <v>45794.878334374996</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>49</v>
       </c>
@@ -4046,7 +4065,7 @@
         <v>45646.883798726849</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>49</v>
       </c>
@@ -4084,7 +4103,7 @@
         <v>45699.641425578702</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
         <v>49</v>
       </c>
@@ -4128,7 +4147,7 @@
         <v>45794.878587500003</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" s="7" t="s">
         <v>63</v>
       </c>
@@ -4166,7 +4185,7 @@
         <v>45794.878587500003</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" s="7" t="s">
         <v>63</v>
       </c>
@@ -4204,7 +4223,7 @@
         <v>45794.761007754627</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
         <v>49</v>
       </c>
@@ -4242,7 +4261,7 @@
         <v>45661.897263078703</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
         <v>49</v>
       </c>
@@ -4283,7 +4302,7 @@
         <v>45795.005495370373</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
         <v>49</v>
       </c>
@@ -4321,7 +4340,7 @@
         <v>45794.759724768519</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
         <v>49</v>
       </c>
@@ -4359,7 +4378,7 @@
         <v>45794.941684722224</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
         <v>49</v>
       </c>
@@ -4397,7 +4416,7 @@
         <v>45794.900951041665</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
         <v>49</v>
       </c>
@@ -4435,7 +4454,7 @@
         <v>45794.879682870371</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>49</v>
       </c>
@@ -4473,7 +4492,7 @@
         <v>45795.000866319446</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
         <v>49</v>
       </c>
@@ -4511,7 +4530,7 @@
         <v>45794.934243055555</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
         <v>49</v>
       </c>
@@ -4549,7 +4568,7 @@
         <v>45794.934243055555</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
         <v>49</v>
       </c>
@@ -4587,7 +4606,7 @@
         <v>45794.934243055555</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
         <v>49</v>
       </c>
@@ -4625,7 +4644,7 @@
         <v>45794.998487847224</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
         <v>49</v>
       </c>
@@ -4663,7 +4682,7 @@
         <v>45794.998487847224</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
         <v>49</v>
       </c>
@@ -4701,7 +4720,7 @@
         <v>45794.998487847224</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
         <v>49</v>
       </c>
@@ -4742,7 +4761,7 @@
         <v>45795.012799074073</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
         <v>49</v>
       </c>
@@ -4780,7 +4799,7 @@
         <v>45795.005366666664</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
         <v>49</v>
       </c>
@@ -4818,7 +4837,7 @@
         <v>45794.895426273149</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
         <v>49</v>
       </c>
@@ -4856,7 +4875,7 @@
         <v>45795.005954282409</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
         <v>49</v>
       </c>
@@ -4894,7 +4913,7 @@
         <v>45794.88801412037</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
         <v>49</v>
       </c>
@@ -4932,7 +4951,7 @@
         <v>45794.88801412037</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
         <v>49</v>
       </c>
@@ -4970,7 +4989,7 @@
         <v>45794.88801412037</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
         <v>49</v>
       </c>
@@ -5008,7 +5027,7 @@
         <v>45794.88801412037</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
         <v>49</v>
       </c>
@@ -5043,7 +5062,7 @@
         <v>45795.013092476853</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
         <v>49</v>
       </c>
@@ -5081,7 +5100,7 @@
         <v>45794.88801412037</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
         <v>49</v>
       </c>
@@ -5116,7 +5135,7 @@
         <v>45795.013152777778</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
         <v>49</v>
       </c>
@@ -5154,7 +5173,7 @@
         <v>45794.996764120369</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
         <v>49</v>
       </c>
@@ -5192,7 +5211,7 @@
         <v>45798.956146180557</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
         <v>49</v>
       </c>
@@ -5233,7 +5252,7 @@
         <v>45794.88801412037</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
         <v>49</v>
       </c>
@@ -5277,7 +5296,7 @@
         <v>45795.004241550923</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
         <v>49</v>
       </c>
@@ -5318,7 +5337,7 @@
         <v>45795.004385532404</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
         <v>49</v>
       </c>
@@ -5362,7 +5381,7 @@
         <v>45794.921978819446</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
         <v>49</v>
       </c>
@@ -5400,7 +5419,7 @@
         <v>45809.837934374998</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
         <v>49</v>
       </c>
@@ -5438,7 +5457,7 @@
         <v>45794.996380555553</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
         <v>49</v>
       </c>
@@ -5476,7 +5495,7 @@
         <v>45794.88801412037</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
         <v>49</v>
       </c>
@@ -5517,7 +5536,7 @@
         <v>45795.006290509256</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
         <v>49</v>
       </c>
@@ -5558,7 +5577,7 @@
         <v>45643.709466666667</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
         <v>49</v>
       </c>
@@ -5602,7 +5621,7 @@
         <v>45642.605838310184</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
         <v>49</v>
       </c>
@@ -5643,7 +5662,7 @@
         <v>45643.709010995372</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
         <v>49</v>
       </c>
@@ -5687,7 +5706,7 @@
         <v>45794.999953935185</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
         <v>49</v>
       </c>
@@ -5728,7 +5747,7 @@
         <v>45794.983736458336</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
         <v>49</v>
       </c>
@@ -5766,7 +5785,7 @@
         <v>45795.012884837961</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A112" s="5" t="s">
         <v>49</v>
       </c>
@@ -5807,7 +5826,7 @@
         <v>45643.705772337962</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
         <v>49</v>
       </c>
@@ -5845,7 +5864,7 @@
         <v>45643.707148842594</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
         <v>49</v>
       </c>
@@ -5883,7 +5902,7 @@
         <v>45643.699993402777</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
         <v>49</v>
       </c>
@@ -5927,7 +5946,7 @@
         <v>45663.844060416668</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
         <v>49</v>
       </c>
@@ -5968,7 +5987,7 @@
         <v>45663.844104976852</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
         <v>49</v>
       </c>
@@ -6009,7 +6028,7 @@
         <v>45795.502180208336</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A118" s="5" t="s">
         <v>49</v>
       </c>
@@ -6044,7 +6063,7 @@
         <v>45798.646983333332</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A119" s="5" t="s">
         <v>49</v>
       </c>
@@ -6076,7 +6095,7 @@
         <v>45798.645414004626</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A120" s="5" t="s">
         <v>49</v>
       </c>
@@ -6114,982 +6133,982 @@
         <v>45794.746116550923</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M121"/>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M122"/>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M123"/>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M124"/>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M125"/>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M126"/>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M127"/>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M128"/>
     </row>
-    <row r="129" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="129" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M129"/>
     </row>
-    <row r="130" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="130" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M130"/>
     </row>
-    <row r="131" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="131" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M131"/>
     </row>
-    <row r="132" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="132" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M132"/>
     </row>
-    <row r="133" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="133" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M133"/>
     </row>
-    <row r="134" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="134" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M134"/>
     </row>
-    <row r="135" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="135" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M135"/>
     </row>
-    <row r="136" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="136" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M136"/>
     </row>
-    <row r="137" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="137" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M137"/>
     </row>
-    <row r="138" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="138" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M138"/>
     </row>
-    <row r="139" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="139" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M139"/>
     </row>
-    <row r="140" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="140" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M140"/>
     </row>
-    <row r="141" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="141" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M141"/>
     </row>
-    <row r="142" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="142" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M142"/>
     </row>
-    <row r="143" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="143" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M143"/>
     </row>
-    <row r="144" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="144" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M144"/>
     </row>
-    <row r="145" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="145" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M145"/>
     </row>
-    <row r="146" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="146" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M146"/>
     </row>
-    <row r="147" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="147" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M147"/>
     </row>
-    <row r="148" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="148" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M148"/>
     </row>
-    <row r="149" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="149" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M149"/>
     </row>
-    <row r="150" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="150" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M150"/>
     </row>
-    <row r="151" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="151" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M151"/>
     </row>
-    <row r="152" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="152" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M152"/>
     </row>
-    <row r="153" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="153" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M153"/>
     </row>
-    <row r="154" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="154" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M154"/>
     </row>
-    <row r="155" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="155" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M155"/>
     </row>
-    <row r="156" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="156" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M156"/>
     </row>
-    <row r="157" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="157" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M157"/>
     </row>
-    <row r="158" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="158" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M158"/>
     </row>
-    <row r="159" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="159" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M159"/>
     </row>
-    <row r="160" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="160" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M160"/>
     </row>
-    <row r="161" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="161" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M161"/>
     </row>
-    <row r="162" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="162" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M162"/>
     </row>
-    <row r="163" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="163" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M163"/>
     </row>
-    <row r="164" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="164" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M164"/>
     </row>
-    <row r="165" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="165" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M165"/>
     </row>
-    <row r="166" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="166" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M166"/>
     </row>
-    <row r="167" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="167" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M167"/>
     </row>
-    <row r="168" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="168" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M168"/>
     </row>
-    <row r="169" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="169" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M169"/>
     </row>
-    <row r="170" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="170" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M170"/>
     </row>
-    <row r="171" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="171" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M171"/>
     </row>
-    <row r="172" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="172" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M172"/>
     </row>
-    <row r="173" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="173" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M173"/>
     </row>
-    <row r="174" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="174" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M174"/>
     </row>
-    <row r="175" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="175" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M175"/>
     </row>
-    <row r="176" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="176" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M176"/>
     </row>
-    <row r="177" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="177" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M177"/>
     </row>
-    <row r="178" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="178" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M178"/>
     </row>
-    <row r="179" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="179" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M179"/>
     </row>
-    <row r="180" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="180" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M180"/>
     </row>
-    <row r="181" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="181" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M181"/>
     </row>
-    <row r="182" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="182" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M182"/>
     </row>
-    <row r="183" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="183" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M183"/>
     </row>
-    <row r="184" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="184" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M184"/>
     </row>
-    <row r="185" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="185" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M185"/>
     </row>
-    <row r="186" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="186" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M186"/>
     </row>
-    <row r="187" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="187" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M187"/>
     </row>
-    <row r="188" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="188" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M188"/>
     </row>
-    <row r="189" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="189" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M189"/>
     </row>
-    <row r="190" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="190" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M190"/>
     </row>
-    <row r="191" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="191" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M191"/>
     </row>
-    <row r="192" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="192" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M192"/>
     </row>
-    <row r="193" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="193" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M193"/>
     </row>
-    <row r="194" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="194" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M194"/>
     </row>
-    <row r="195" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="195" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M195"/>
     </row>
-    <row r="196" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="196" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M196"/>
     </row>
-    <row r="197" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="197" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M197"/>
     </row>
-    <row r="198" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="198" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M198"/>
     </row>
-    <row r="199" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="199" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M199"/>
     </row>
-    <row r="200" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="200" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M200"/>
     </row>
-    <row r="201" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="201" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M201"/>
     </row>
-    <row r="202" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="202" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M202"/>
     </row>
-    <row r="203" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="203" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M203"/>
     </row>
-    <row r="204" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="204" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M204"/>
     </row>
-    <row r="205" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="205" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M205"/>
     </row>
-    <row r="206" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="206" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M206"/>
     </row>
-    <row r="207" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="207" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M207"/>
     </row>
-    <row r="208" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="208" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M208"/>
     </row>
-    <row r="209" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="209" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M209"/>
     </row>
-    <row r="210" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="210" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M210"/>
     </row>
-    <row r="211" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="211" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M211"/>
     </row>
-    <row r="212" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="212" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M212"/>
     </row>
-    <row r="213" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="213" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M213"/>
     </row>
-    <row r="214" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="214" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M214"/>
     </row>
-    <row r="215" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="215" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M215"/>
     </row>
-    <row r="216" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="216" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M216"/>
     </row>
-    <row r="217" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="217" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M217"/>
     </row>
-    <row r="218" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="218" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M218"/>
     </row>
-    <row r="219" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="219" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M219"/>
     </row>
-    <row r="220" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="220" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M220"/>
     </row>
-    <row r="221" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="221" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M221"/>
     </row>
-    <row r="222" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="222" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M222"/>
     </row>
-    <row r="223" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="223" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M223"/>
     </row>
-    <row r="224" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="224" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M224"/>
     </row>
-    <row r="225" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="225" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M225"/>
     </row>
-    <row r="226" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="226" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M226"/>
     </row>
-    <row r="227" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="227" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M227"/>
     </row>
-    <row r="228" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="228" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M228"/>
     </row>
-    <row r="229" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="229" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M229"/>
     </row>
-    <row r="230" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="230" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M230"/>
     </row>
-    <row r="231" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="231" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M231"/>
     </row>
-    <row r="232" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="232" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M232"/>
     </row>
-    <row r="233" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="233" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M233"/>
     </row>
-    <row r="234" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="234" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M234"/>
     </row>
-    <row r="235" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="235" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M235"/>
     </row>
-    <row r="236" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="236" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M236"/>
     </row>
-    <row r="237" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="237" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M237"/>
     </row>
-    <row r="238" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="238" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M238"/>
     </row>
-    <row r="239" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="239" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M239"/>
     </row>
-    <row r="240" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="240" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M240"/>
     </row>
-    <row r="241" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="241" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M241"/>
     </row>
-    <row r="242" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="242" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M242"/>
     </row>
-    <row r="243" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="243" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M243"/>
     </row>
-    <row r="244" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="244" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M244"/>
     </row>
-    <row r="245" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="245" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M245"/>
     </row>
-    <row r="246" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="246" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M246"/>
     </row>
-    <row r="247" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="247" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M247"/>
     </row>
-    <row r="248" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="248" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M248"/>
     </row>
-    <row r="249" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="249" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M249"/>
     </row>
-    <row r="250" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="250" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M250"/>
     </row>
-    <row r="251" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="251" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M251"/>
     </row>
-    <row r="252" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="252" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M252"/>
     </row>
-    <row r="253" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="253" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M253"/>
     </row>
-    <row r="254" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="254" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M254"/>
     </row>
-    <row r="255" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="255" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M255"/>
     </row>
-    <row r="256" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="256" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M256"/>
     </row>
-    <row r="257" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="257" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M257"/>
     </row>
-    <row r="258" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="258" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M258"/>
     </row>
-    <row r="259" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="259" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M259"/>
     </row>
-    <row r="260" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="260" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M260"/>
     </row>
-    <row r="261" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="261" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M261"/>
     </row>
-    <row r="262" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="262" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M262"/>
     </row>
-    <row r="263" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="263" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M263"/>
     </row>
-    <row r="264" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="264" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M264"/>
     </row>
-    <row r="265" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="265" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M265"/>
     </row>
-    <row r="266" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="266" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M266"/>
     </row>
-    <row r="267" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="267" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M267"/>
     </row>
-    <row r="268" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="268" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M268"/>
     </row>
-    <row r="269" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="269" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M269"/>
     </row>
-    <row r="270" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="270" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M270"/>
     </row>
-    <row r="271" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="271" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M271"/>
     </row>
-    <row r="272" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="272" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M272"/>
     </row>
-    <row r="273" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="273" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M273"/>
     </row>
-    <row r="274" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="274" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M274"/>
     </row>
-    <row r="275" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="275" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M275"/>
     </row>
-    <row r="276" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="276" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M276"/>
     </row>
-    <row r="277" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="277" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M277"/>
     </row>
-    <row r="278" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="278" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M278"/>
     </row>
-    <row r="279" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="279" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M279"/>
     </row>
-    <row r="280" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="280" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M280"/>
     </row>
-    <row r="281" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="281" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M281"/>
     </row>
-    <row r="282" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="282" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M282"/>
     </row>
-    <row r="283" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="283" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M283"/>
     </row>
-    <row r="284" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="284" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M284"/>
     </row>
-    <row r="285" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="285" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M285"/>
     </row>
-    <row r="286" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="286" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M286"/>
     </row>
-    <row r="287" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="287" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M287"/>
     </row>
-    <row r="288" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="288" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M288"/>
     </row>
-    <row r="289" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="289" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M289"/>
     </row>
-    <row r="290" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="290" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M290"/>
     </row>
-    <row r="291" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="291" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M291"/>
     </row>
-    <row r="292" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="292" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M292"/>
     </row>
-    <row r="293" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="293" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M293"/>
     </row>
-    <row r="294" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="294" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M294"/>
     </row>
-    <row r="295" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="295" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M295"/>
     </row>
-    <row r="296" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="296" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M296"/>
     </row>
-    <row r="297" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="297" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M297"/>
     </row>
-    <row r="298" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="298" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M298"/>
     </row>
-    <row r="299" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="299" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M299"/>
     </row>
-    <row r="300" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="300" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M300"/>
     </row>
-    <row r="301" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="301" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M301"/>
     </row>
-    <row r="302" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="302" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M302"/>
     </row>
-    <row r="303" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="303" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M303"/>
     </row>
-    <row r="304" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="304" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M304"/>
     </row>
-    <row r="305" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="305" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M305"/>
     </row>
-    <row r="306" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="306" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M306"/>
     </row>
-    <row r="307" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="307" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M307"/>
     </row>
-    <row r="308" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="308" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M308"/>
     </row>
-    <row r="309" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="309" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M309"/>
     </row>
-    <row r="310" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="310" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M310"/>
     </row>
-    <row r="311" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="311" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M311"/>
     </row>
-    <row r="312" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="312" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M312"/>
     </row>
-    <row r="313" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="313" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M313"/>
     </row>
-    <row r="314" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="314" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M314"/>
     </row>
-    <row r="315" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="315" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M315"/>
     </row>
-    <row r="316" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="316" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M316"/>
     </row>
-    <row r="317" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="317" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M317"/>
     </row>
-    <row r="318" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="318" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M318"/>
     </row>
-    <row r="319" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="319" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M319"/>
     </row>
-    <row r="320" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="320" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M320"/>
     </row>
-    <row r="321" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="321" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M321"/>
     </row>
-    <row r="322" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="322" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M322"/>
     </row>
-    <row r="323" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="323" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M323"/>
     </row>
-    <row r="324" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="324" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M324"/>
     </row>
-    <row r="325" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="325" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M325"/>
     </row>
-    <row r="326" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="326" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M326"/>
     </row>
-    <row r="327" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="327" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M327"/>
     </row>
-    <row r="328" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="328" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M328"/>
     </row>
-    <row r="329" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="329" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M329"/>
     </row>
-    <row r="330" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="330" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M330"/>
     </row>
-    <row r="331" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="331" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M331"/>
     </row>
-    <row r="332" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="332" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M332"/>
     </row>
-    <row r="333" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="333" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M333"/>
     </row>
-    <row r="334" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="334" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M334"/>
     </row>
-    <row r="335" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="335" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M335"/>
     </row>
-    <row r="336" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="336" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M336"/>
     </row>
-    <row r="337" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="337" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M337"/>
     </row>
-    <row r="338" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="338" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M338"/>
     </row>
-    <row r="339" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="339" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M339"/>
     </row>
-    <row r="340" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="340" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M340"/>
     </row>
-    <row r="341" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="341" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M341"/>
     </row>
-    <row r="342" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="342" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M342"/>
     </row>
-    <row r="343" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="343" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M343"/>
     </row>
-    <row r="344" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="344" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M344"/>
     </row>
-    <row r="345" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="345" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M345"/>
     </row>
-    <row r="346" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="346" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M346"/>
     </row>
-    <row r="347" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="347" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M347"/>
     </row>
-    <row r="348" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="348" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M348"/>
     </row>
-    <row r="349" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="349" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M349"/>
     </row>
-    <row r="350" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="350" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M350"/>
     </row>
-    <row r="351" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="351" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M351"/>
     </row>
-    <row r="352" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="352" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M352"/>
     </row>
-    <row r="353" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="353" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M353"/>
     </row>
-    <row r="354" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="354" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M354"/>
     </row>
-    <row r="355" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="355" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M355"/>
     </row>
-    <row r="356" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="356" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M356"/>
     </row>
-    <row r="357" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="357" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M357"/>
     </row>
-    <row r="358" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="358" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M358"/>
     </row>
-    <row r="359" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="359" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M359"/>
     </row>
-    <row r="360" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="360" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M360"/>
     </row>
-    <row r="361" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="361" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M361"/>
     </row>
-    <row r="362" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="362" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M362"/>
     </row>
-    <row r="363" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="363" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M363"/>
     </row>
-    <row r="364" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="364" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M364"/>
     </row>
-    <row r="365" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="365" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M365"/>
     </row>
-    <row r="366" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="366" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M366"/>
     </row>
-    <row r="367" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="367" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M367"/>
     </row>
-    <row r="368" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="368" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M368"/>
     </row>
-    <row r="369" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="369" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M369"/>
     </row>
-    <row r="370" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="370" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M370"/>
     </row>
-    <row r="371" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="371" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M371"/>
     </row>
-    <row r="372" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="372" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M372"/>
     </row>
-    <row r="373" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="373" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M373"/>
     </row>
-    <row r="374" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="374" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M374"/>
     </row>
-    <row r="375" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="375" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M375"/>
     </row>
-    <row r="376" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="376" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M376"/>
     </row>
-    <row r="377" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="377" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M377"/>
     </row>
-    <row r="378" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="378" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M378"/>
     </row>
-    <row r="379" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="379" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M379"/>
     </row>
-    <row r="380" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="380" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M380"/>
     </row>
-    <row r="381" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="381" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M381"/>
     </row>
-    <row r="382" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="382" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M382"/>
     </row>
-    <row r="383" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="383" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M383"/>
     </row>
-    <row r="384" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="384" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M384"/>
     </row>
-    <row r="385" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="385" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M385"/>
     </row>
-    <row r="386" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="386" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M386"/>
     </row>
-    <row r="387" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="387" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M387"/>
     </row>
-    <row r="388" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="388" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M388"/>
     </row>
-    <row r="389" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="389" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M389"/>
     </row>
-    <row r="390" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="390" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M390"/>
     </row>
-    <row r="391" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="391" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M391"/>
     </row>
-    <row r="392" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="392" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M392"/>
     </row>
-    <row r="393" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="393" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M393"/>
     </row>
-    <row r="394" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="394" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M394"/>
     </row>
-    <row r="395" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="395" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M395"/>
     </row>
-    <row r="396" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="396" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M396"/>
     </row>
-    <row r="397" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="397" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M397"/>
     </row>
-    <row r="398" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="398" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M398"/>
     </row>
-    <row r="399" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="399" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M399"/>
     </row>
-    <row r="400" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="400" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M400"/>
     </row>
-    <row r="401" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="401" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M401"/>
     </row>
-    <row r="402" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="402" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M402"/>
     </row>
-    <row r="403" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="403" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M403"/>
     </row>
-    <row r="404" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="404" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M404"/>
     </row>
-    <row r="405" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="405" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M405"/>
     </row>
-    <row r="406" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="406" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M406"/>
     </row>
-    <row r="407" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="407" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M407"/>
     </row>
-    <row r="408" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="408" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M408"/>
     </row>
-    <row r="409" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="409" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M409"/>
     </row>
-    <row r="410" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="410" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M410"/>
     </row>
-    <row r="411" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="411" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M411"/>
     </row>
-    <row r="412" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="412" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M412"/>
     </row>
-    <row r="413" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="413" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M413"/>
     </row>
-    <row r="414" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="414" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M414"/>
     </row>
-    <row r="415" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="415" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M415"/>
     </row>
-    <row r="416" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="416" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M416"/>
     </row>
-    <row r="417" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="417" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M417"/>
     </row>
-    <row r="418" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="418" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M418"/>
     </row>
-    <row r="419" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="419" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M419"/>
     </row>
-    <row r="420" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="420" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M420"/>
     </row>
-    <row r="421" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="421" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M421"/>
     </row>
-    <row r="422" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="422" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M422"/>
     </row>
-    <row r="423" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="423" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M423"/>
     </row>
-    <row r="424" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="424" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M424"/>
     </row>
-    <row r="425" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="425" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M425"/>
     </row>
-    <row r="426" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="426" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M426"/>
     </row>
-    <row r="427" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="427" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M427"/>
     </row>
-    <row r="428" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="428" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M428"/>
     </row>
-    <row r="429" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="429" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M429"/>
     </row>
-    <row r="430" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="430" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M430"/>
     </row>
-    <row r="431" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="431" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M431"/>
     </row>
-    <row r="432" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="432" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M432"/>
     </row>
-    <row r="433" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="433" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M433"/>
     </row>
-    <row r="434" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="434" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M434"/>
     </row>
-    <row r="435" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="435" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M435"/>
     </row>
-    <row r="436" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="436" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M436"/>
     </row>
-    <row r="437" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="437" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M437"/>
     </row>
-    <row r="438" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="438" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M438"/>
     </row>
-    <row r="439" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="439" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M439"/>
     </row>
-    <row r="440" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="440" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M440"/>
     </row>
-    <row r="441" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="441" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M441"/>
     </row>
-    <row r="442" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="442" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M442"/>
     </row>
-    <row r="443" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="443" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M443"/>
     </row>
-    <row r="444" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="444" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M444"/>
     </row>
-    <row r="445" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="445" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M445"/>
     </row>
-    <row r="446" spans="13:13" x14ac:dyDescent="0.45">
+    <row r="446" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M446"/>
     </row>
   </sheetData>
@@ -7207,13 +7226,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84D39259-A685-447E-BA98-114E78E460C1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.265625" customWidth="1"/>
-    <col min="5" max="5" width="12.59765625" customWidth="1"/>
+    <col min="1" max="1" width="29.21875" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>309</v>
       </c>
@@ -7222,7 +7241,7 @@
         <v>496.6</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -7234,7 +7253,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>310</v>
       </c>
@@ -7246,7 +7265,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>312</v>
       </c>
@@ -7266,12 +7285,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B74596AE-BA65-43C6-BFB1-FEC7E7BCF1F4}">
   <dimension ref="E9:G20"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="19.1328125" customWidth="1"/>
+    <col min="5" max="5" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="5:7" x14ac:dyDescent="0.45">
+    <row r="9" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
         <v>155</v>
       </c>
@@ -7282,7 +7301,7 @@
         <v>9.99</v>
       </c>
     </row>
-    <row r="12" spans="5:7" x14ac:dyDescent="0.45">
+    <row r="12" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
         <v>184</v>
       </c>
@@ -7293,7 +7312,7 @@
         <v>9.99</v>
       </c>
     </row>
-    <row r="13" spans="5:7" x14ac:dyDescent="0.45">
+    <row r="13" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E13" t="s">
         <v>185</v>
       </c>
@@ -7304,7 +7323,7 @@
         <v>18.989999999999998</v>
       </c>
     </row>
-    <row r="15" spans="5:7" x14ac:dyDescent="0.45">
+    <row r="15" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E15" t="s">
         <v>247</v>
       </c>
@@ -7315,7 +7334,7 @@
         <v>11.79</v>
       </c>
     </row>
-    <row r="17" spans="5:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
         <v>253</v>
       </c>
@@ -7326,7 +7345,7 @@
         <v>17.989999999999998</v>
       </c>
     </row>
-    <row r="20" spans="5:7" x14ac:dyDescent="0.45">
+    <row r="20" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
         <v>292</v>
       </c>
@@ -7353,12 +7372,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33E5102B-C60B-45F7-99D3-4FD643D162CB}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="25.59765625" customWidth="1"/>
+    <col min="2" max="2" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -7366,7 +7385,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>67</v>
       </c>
@@ -7374,7 +7393,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>129</v>
       </c>
@@ -7382,7 +7401,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>250</v>
       </c>
@@ -7390,7 +7409,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>85</v>
       </c>
@@ -7398,7 +7417,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>302</v>
       </c>
@@ -7412,11 +7431,50 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0671F1B1-02F0-4EC7-9647-526F8564CDB4}">
+  <dimension ref="D10:E12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="10" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>317</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="11" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>319</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="12" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>321</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E10" r:id="rId1" xr:uid="{8C91DDA8-6DDE-4293-A231-4E6E0E4F3B1B}"/>
+    <hyperlink ref="E11" r:id="rId2" xr:uid="{23BB51DB-162D-4559-992A-23C35A9800EB}"/>
+    <hyperlink ref="E12" r:id="rId3" xr:uid="{9F272314-EBAC-41E5-804B-8CA6733FD934}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CC74B92-87B0-4A22-A923-4C67B6D818A0}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>305</v>
       </c>

</xml_diff>